<commit_message>
Convert the active schedule per personnel number
Pin calendar-conversion v0.3.0 and add a scope parameter to the active
schedule conversion: personal (the default) returns the caller's events
plus the events for everyone, and full returns the whole schedule for a
super_user only. An account without a personnel number gets
409 missing_personnel_number. The converter page gives a super_user a
"Nur meine Termine" toggle, blocks an account without a number, and shows
a neutral message when the schedule has no events for the caller. The
example schedule gains a participants column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/examples/calendar_schedule_example.xlsx
+++ b/assets/examples/calendar_schedule_example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paolorossi/Develop/firefighter-app-ui/assets/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08D9385-1504-6F45-BE79-C388916C2AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBBFC468-556F-4E42-9B46-4FC0F05E09BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="620" windowWidth="33720" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>id</t>
   </si>
@@ -49,16 +49,43 @@
     <t>description</t>
   </si>
   <si>
+    <t>participants</t>
+  </si>
+  <si>
+    <t>dienst-2026-08-08</t>
+  </si>
+  <si>
+    <t>Bereitschaftsdienst</t>
+  </si>
+  <si>
     <t>Feuerwehrhaus</t>
   </si>
   <si>
-    <t>dienst-2026-08-08</t>
-  </si>
-  <si>
-    <t>Bereitschaftsdienst</t>
-  </si>
-  <si>
     <t>Ganztägiger Dienst</t>
+  </si>
+  <si>
+    <t>uebung-2026-08-12</t>
+  </si>
+  <si>
+    <t>Atemschutzübung</t>
+  </si>
+  <si>
+    <t>Übung der Atemschutzträger</t>
+  </si>
+  <si>
+    <t>nachtdienst-2026-08-15</t>
+  </si>
+  <si>
+    <t>Nachtdienst</t>
+  </si>
+  <si>
+    <t>Nachtbereitschaft</t>
+  </si>
+  <si>
+    <t>101;202</t>
+  </si>
+  <si>
+    <t>202</t>
   </si>
 </sst>
 </file>
@@ -136,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -146,11 +173,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -160,6 +182,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -176,23 +201,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <bag type="Checkbox"/>
-  <bag type="XFControls">
-    <bagId k="CellControl">0</bagId>
-  </bag>
-  <bag type="XFComplement">
-    <bagId k="XFControls">1</bagId>
-  </bag>
-  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
-</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -390,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -402,9 +410,10 @@
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28" customHeight="1">
+    <row r="1" spans="1:10" ht="28" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,8 +441,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="23" customHeight="1">
+    <row r="2" spans="1:10" ht="23" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -452,10 +464,75 @@
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="7"/>
+    </row>
+    <row r="3" spans="1:10" ht="16">
+      <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>46246</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F3" s="4">
+        <v>46246</v>
+      </c>
+      <c r="G3" s="5">
+        <v>0.875</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>12</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="16">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>46249</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F4" s="4">
+        <v>46250</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>